<commit_message>
Add numeric-aware diffs, recursive table discovery, and Change Log Detail.csv sidecar.
Preserve dummy lines and encoding fallback, and refresh acceptance fixtures and docs to match the new Stage 1/2 behavior.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/fixtures/acceptance/T01_two_crs_no_overlap/Output/ChangeLog_T01_RUN.xlsx
+++ b/fixtures/acceptance/T01_two_crs_no_overlap/Output/ChangeLog_T01_RUN.xlsx
@@ -8,10 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChangeLog_Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXPENSE_TABLE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MORT_TABLE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXPENSE_TABLE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MORT_TABLE" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -585,13 +584,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>change_request_id</t>
+          <t>conflict_type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -601,132 +600,44 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>change_type</t>
+          <t>key_tuple</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>n_keys_before</t>
+          <t>column_name</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>n_keys_after</t>
+          <t>change_request_ids</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>key_tuple</t>
+          <t>change_types</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>column_name</t>
+          <t>old_values</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>old_value</t>
+          <t>new_values</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>new_value</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CR_T01_Mortality</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>MORT_TABLE</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>value_update</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>20|1|PROD_A</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>0.0012</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.0013</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CR_T01_Expense</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>EXPENSE_TABLE</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>value_update</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PROD_A|ACQ</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>resolved</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -739,58 +650,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>conflict_type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>table_name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>key_tuple</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>column_name</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>change_request_ids</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>change_types</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>old_values</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>new_values</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>resolved</t>
+          <t>Review: EXPENSE_TABLE (human review only - not used by apply)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>_change</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ExpenseType</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[CR_T01_Expense]</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROD_A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ACQ</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>100 -&gt; 110</t>
         </is>
       </c>
     </row>
@@ -805,13 +715,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Review: EXPENSE_TABLE (human review only - not used by apply)</t>
+          <t>Review: MORT_TABLE (human review only - not used by apply)</t>
         </is>
       </c>
     </row>
@@ -823,144 +733,51 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>ExpenseType</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Amount</t>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Loading</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[CR_T01_Mortality]</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>PROD_A</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ACQ</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>100 -&gt; 110</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PROD_A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>MAINT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PROD_B</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ACQ</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Review: MORT_TABLE (human review only - not used by apply)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>_change</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Duration</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>PROD_A</t>
-        </is>
-      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>0.0012 -&gt; 0.0013</t>
@@ -969,62 +786,6 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>1.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>PROD_A</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.0015</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>PROD_B</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0.0020</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1.10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split Change Log reviews into per-folder workbooks and apply Stage 2 changes sequentially in Control order so later CRs see earlier results.
Pin Polars 1.44.2, prompt for an optional Change Log in Run.bat, and refresh docs, UML, and acceptance fixtures.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/fixtures/acceptance/T01_two_crs_no_overlap/Output/ChangeLog_T01_RUN.xlsx
+++ b/fixtures/acceptance/T01_two_crs_no_overlap/Output/ChangeLog_T01_RUN.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXPENSE_TABLE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MORT_TABLE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReviewFiles" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,24 +31,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,11 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -650,142 +635,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Review: EXPENSE_TABLE (human review only - not used by apply)</t>
+          <t>table_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>review_file</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EXPENSE_TABLE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ChangeLog_T01_RUN_reviews/root.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>_change</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>ExpenseType</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>[CR_T01_Expense]</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PROD_A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ACQ</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>100 -&gt; 110</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Review: MORT_TABLE (human review only - not used by apply)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>_change</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Duration</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Loading</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>[CR_T01_Mortality]</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>PROD_A</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>0.0012 -&gt; 0.0013</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1.05</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MORT_TABLE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ChangeLog_T01_RUN_reviews/root.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>